<commit_message>
Adding New Projects and files
</commit_message>
<xml_diff>
--- a/Omega_Industries_Indirect_CFS.xlsx
+++ b/Omega_Industries_Indirect_CFS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/azrael/Desktop/365 finance/fundamentals-of-financial-reporting/Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/azrael/Desktop/my-portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80C049CC-761C-BA43-8F24-248C3DE23981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E879DE22-693F-1F42-A615-D2B6538E59F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" tabRatio="854" activeTab="4" xr2:uid="{9FC57020-DF4D-4BD6-8F0A-F8AA1857DDAF}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" tabRatio="854" activeTab="4" xr2:uid="{9FC57020-DF4D-4BD6-8F0A-F8AA1857DDAF}"/>
   </bookViews>
   <sheets>
     <sheet name="Income Statement" sheetId="1" r:id="rId1"/>
@@ -894,6 +894,15 @@
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -903,15 +912,6 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2599,7 +2599,7 @@
         <v>-10248</v>
       </c>
       <c r="D17" s="54"/>
-      <c r="E17" s="73" t="s">
+      <c r="E17" s="82" t="s">
         <v>107</v>
       </c>
       <c r="F17" s="62"/>
@@ -2613,7 +2613,7 @@
         <v>22142</v>
       </c>
       <c r="D18" s="54"/>
-      <c r="E18" s="74"/>
+      <c r="E18" s="83"/>
       <c r="F18" s="62"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.15">
@@ -2625,7 +2625,7 @@
         <v>-24731</v>
       </c>
       <c r="D19" s="54"/>
-      <c r="E19" s="75"/>
+      <c r="E19" s="84"/>
       <c r="F19" s="62"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.15">
@@ -2795,7 +2795,7 @@
     </row>
     <row r="41" spans="2:6" ht="13" thickTop="1" x14ac:dyDescent="0.15"/>
     <row r="42" spans="2:6" x14ac:dyDescent="0.15">
-      <c r="B42" s="76" t="s">
+      <c r="B42" s="73" t="s">
         <v>73</v>
       </c>
       <c r="C42" s="54">
@@ -2857,7 +2857,7 @@
         <f>C11+C14+C10*(1-0.2)+SUM(C17:C19)+SUM(C30:C31)</f>
         <v>3913</v>
       </c>
-      <c r="E49" s="83" t="str">
+      <c r="E49" s="80" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C49)</f>
         <v>=C11+C14+C10*(1-0.2)+SUM(C17:C19)+SUM(C30:C31)</v>
       </c>
@@ -2870,7 +2870,7 @@
         <f>C22+SUM(C30:C31)+C10*(1-0.2)</f>
         <v>3913</v>
       </c>
-      <c r="E50" s="84" t="str">
+      <c r="E50" s="81" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C50)</f>
         <v>=C22+SUM(C30:C31)+C10*(1-0.2)</v>
       </c>
@@ -2887,7 +2887,7 @@
         <f>C22+C32+C38</f>
         <v>-2330</v>
       </c>
-      <c r="E52" s="83" t="str">
+      <c r="E52" s="80" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C52)</f>
         <v>=C22+C32+C38</v>
       </c>
@@ -2900,7 +2900,7 @@
         <f>C50+C25*(1-0.2)+C38</f>
         <v>-2330</v>
       </c>
-      <c r="E53" s="84" t="str">
+      <c r="E53" s="81" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C53)</f>
         <v>=C50+C25*(1-0.2)+C38</v>
       </c>
@@ -2913,38 +2913,38 @@
       </c>
     </row>
     <row r="56" spans="2:6" x14ac:dyDescent="0.15">
-      <c r="B56" s="79" t="s">
+      <c r="B56" s="76" t="s">
         <v>114</v>
       </c>
-      <c r="C56" s="77"/>
-      <c r="D56" s="77"/>
-      <c r="E56" s="77"/>
-      <c r="F56" s="81"/>
+      <c r="C56" s="74"/>
+      <c r="D56" s="74"/>
+      <c r="E56" s="74"/>
+      <c r="F56" s="78"/>
     </row>
     <row r="57" spans="2:6" x14ac:dyDescent="0.15">
-      <c r="B57" s="80" t="s">
+      <c r="B57" s="77" t="s">
         <v>117</v>
       </c>
-      <c r="C57" s="78"/>
-      <c r="D57" s="78"/>
-      <c r="E57" s="78"/>
-      <c r="F57" s="82"/>
+      <c r="C57" s="75"/>
+      <c r="D57" s="75"/>
+      <c r="E57" s="75"/>
+      <c r="F57" s="79"/>
     </row>
     <row r="59" spans="2:6" x14ac:dyDescent="0.15">
-      <c r="B59" s="79" t="s">
+      <c r="B59" s="76" t="s">
         <v>115</v>
       </c>
-      <c r="C59" s="77"/>
-      <c r="D59" s="77"/>
-      <c r="E59" s="81"/>
+      <c r="C59" s="74"/>
+      <c r="D59" s="74"/>
+      <c r="E59" s="78"/>
     </row>
     <row r="60" spans="2:6" x14ac:dyDescent="0.15">
-      <c r="B60" s="80" t="s">
+      <c r="B60" s="77" t="s">
         <v>116</v>
       </c>
-      <c r="C60" s="78"/>
-      <c r="D60" s="78"/>
-      <c r="E60" s="82"/>
+      <c r="C60" s="75"/>
+      <c r="D60" s="75"/>
+      <c r="E60" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2955,6 +2955,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100382E84A263CF1945AD4232D5B4111E63" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="82926c85b40558f05a495d75f0ef2ab5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="a33b3d48-4748-415e-9501-e406a79056a5" xmlns:ns4="b90b3ce1-30c3-4251-9b85-7842ce11cfd6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="325293254555ca9b253aecf98e7d6abd" ns3:_="" ns4:_="">
     <xsd:import namespace="a33b3d48-4748-415e-9501-e406a79056a5"/>
@@ -3177,22 +3192,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70F813C4-B67D-4800-A177-EEBFAD7DF805}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32DBC92B-9045-4ED1-A176-96595D8365AC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02DD16F4-B7E1-47E6-B3C3-95275B43C434}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3209,21 +3226,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32DBC92B-9045-4ED1-A176-96595D8365AC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70F813C4-B67D-4800-A177-EEBFAD7DF805}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>